<commit_message>
Remove Unit 1 coding questions, fix generic filler descriptions in Unit 2
Per Jul 9 meeting feedback: Unit 1 shouldn't have coding questions, so all
40 are removed. In Unit 2, 10 of 40 questions had placeholder descriptions
("A supplemental Python practice task...") that never stated the actual
rule or formula needed to solve them; rewrote each with a real scenario
and the explicit logic, verified against existing solutions/test cases.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/Question Bank/Coding Questions/Unit 2 - Data Types and Operators/Unit 2 - Data Types and Operators - Coding Questions.xlsx
+++ b/content/Question Bank/Coding Questions/Unit 2 - Data Types and Operators/Unit 2 - Data Types and Operators - Coding Questions.xlsx
@@ -1948,16 +1948,19 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>A supplemental Python practice task for GST Bill Total. Read the input values and print the required result exactly.
+          <t>A grocery store's billing counter needs to add GST to every purchase before printing the final amount on the receipt. GST here is a flat 18 percent of the item's price.
+Write a program that reads the price of an item as a decimal number and prints the final amount after adding 18 percent GST, rounded to exactly two decimal places.
 ### Input Format
-- Line 1: Amount
+- Line 1: Price of the item
 ### Output Format
 ```
 118.0
 ```
+### Example Walkthrough
+In the sample, the price is 100. The GST is 100 x 18 / 100 = 18, so the final amount is 100 + 18 = 118.0.
 ### Constraints
-- Inputs follow the described format.
-- Print exactly the requested output with no extra text.</t>
+- All numeric inputs are valid numbers in the ranges implied by the examples.
+- Every value must be printed exactly as shown in the output format, with no extra text added or removed.</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -2102,16 +2105,19 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>A supplemental Python practice task for Minutes Split. Read the input values and print the required result exactly.
+          <t>A bus tracking app receives a trip's duration in total minutes from the GPS unit, but displays it to passengers in hours and minutes so it is easier to read.
+Write a program that reads the trip duration in minutes as a whole number and prints it split into hours and remaining minutes, in the form `&lt;hours&gt; hours &lt;minutes&gt; minutes`.
 ### Input Format
-- Line 1: Minutes
+- Line 1: Duration in minutes
 ### Output Format
 ```
 2 hours 5 minutes
 ```
+### Example Walkthrough
+In the sample, the duration is 125 minutes. Dividing by 60 gives 2 whole hours (120 minutes), leaving a remainder of 5 minutes, so the program prints `2 hours 5 minutes`.
 ### Constraints
-- Inputs follow the described format.
-- Print exactly the requested output with no extra text.</t>
+- All numeric inputs are valid whole numbers in the ranges implied by the examples.
+- Every value must be printed exactly as shown in the output format, with no extra text added or removed.</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -3794,7 +3800,8 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>A supplemental Python practice task for Name Age Line. Read the input values and print the required result exactly.
+          <t>The college attendance kiosk prints a one-line summary for every student who taps their ID card, combining their name and age into a single readable sentence.
+Write a program that reads a student's name and age, then prints a line in the form `&lt;name&gt; is &lt;age&gt; years old`.
 ### Input Format
 - Line 1: Name
 - Line 2: Age
@@ -3802,9 +3809,11 @@
 ```
 Asha is 19 years old
 ```
+### Example Walkthrough
+In the sample, the name is Asha and the age is 19, so the program prints `Asha is 19 years old`.
 ### Constraints
-- Inputs follow the described format.
-- Print exactly the requested output with no extra text.</t>
+- Name is a valid string with no leading or trailing spaces.
+- Every value must be printed exactly as shown in the output format, with no extra text added or removed.</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -3957,18 +3966,21 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>A supplemental Python practice task for Remainder Counter. Read the input values and print the required result exactly.
+          <t>A warehouse worker is packing items into boxes that each hold a fixed number of items. Before sealing the shipment, the packing software needs to report how many full boxes were made and how many items are left over.
+Write a program that reads the total number of items and the box size, then prints the number of full boxes and the number of leftover items on separate lines.
 ### Input Format
-- Line 1: Items
-- Line 2: Group size
+- Line 1: Total number of items
+- Line 2: Box size
 ### Output Format
 ```
 Full groups: 3
 Left over: 2
 ```
+### Example Walkthrough
+In the sample, there are 17 items and each box holds 5. Dividing gives 17 // 5 = 3 full boxes, with 17 % 5 = 2 items left over, so the program prints `Full groups: 3` and `Left over: 2`.
 ### Constraints
-- Inputs follow the described format.
-- Print exactly the requested output with no extra text.</t>
+- All numeric inputs are valid whole numbers in the ranges implied by the examples.
+- Every value must be printed exactly as shown in the output format, with no extra text added or removed.</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -5564,17 +5576,20 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>A supplemental Python practice task for Compare Scores. Read the input values and print the required result exactly.
+          <t>A sports quiz app wants to instantly tell which of two contestants scored higher, so it can highlight the round's leader on screen.
+Write a program that reads two scores and prints `True` if the first score is strictly greater than the second, and `False` otherwise.
 ### Input Format
-- Line 1: First
-- Line 2: Second
+- Line 1: First score
+- Line 2: Second score
 ### Output Format
 ```
 True
 ```
+### Example Walkthrough
+In the sample, the first score is 90 and the second is 80. Since 90 is greater than 80, the program prints `True`.
 ### Constraints
-- Inputs follow the described format.
-- Print exactly the requested output with no extra text.</t>
+- All numeric inputs are valid whole numbers in the ranges implied by the examples.
+- Every value must be printed exactly as shown in the output format, with no extra text added or removed.</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -5727,17 +5742,20 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>A supplemental Python practice task for Discount Price. Read the input values and print the required result exactly.
+          <t>An online store applies a seasonal discount to every product at checkout, and the app needs to show the discounted price instantly once the customer enters the discount code.
+Write a program that reads the original price and the discount percentage, then prints the price after the discount is applied, rounded to exactly two decimal places.
 ### Input Format
-- Line 1: Price
-- Line 2: Discount percent
+- Line 1: Original price
+- Line 2: Discount percentage
 ### Output Format
 ```
 90.0
 ```
+### Example Walkthrough
+In the sample, the price is 100 with a 10 percent discount. The discount amount is 100 x 10 / 100 = 10, so the final price is 100 - 10 = 90.0.
 ### Constraints
-- Inputs follow the described format.
-- Print exactly the requested output with no extra text.</t>
+- All numeric inputs are valid numbers in the ranges implied by the examples.
+- Every value must be printed exactly as shown in the output format, with no extra text added or removed.</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -5890,7 +5908,8 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>A supplemental Python practice task for Precedence Value. Read the input values and print the required result exactly.
+          <t>A quiz app calculates a player's final score as a base score plus a bonus, where the bonus is the number of bonus questions answered correctly multiplied by the points awarded per bonus question. The app computes this directly as `a + b * c`, relying on Python evaluating multiplication before addition.
+Write a program that reads three whole numbers `a`, `b`, and `c`, then prints the value of the expression `a + b * c`.
 ### Input Format
 - Line 1: a
 - Line 2: b
@@ -5899,9 +5918,11 @@
 ```
 14
 ```
+### Example Walkthrough
+In the sample, a is 2, b is 3, and c is 4. Because multiplication happens before addition, the expression evaluates as 2 + (3 x 4) = 2 + 12 = 14.
 ### Constraints
-- Inputs follow the described format.
-- Print exactly the requested output with no extra text.</t>
+- All numeric inputs are valid whole numbers in the ranges implied by the examples.
+- Every value must be printed exactly as shown in the output format, with no extra text added or removed.</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -7658,18 +7679,21 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>A supplemental Python practice task for Wallet Update. Read the input values and print the required result exactly.
+          <t>A digital wallet app processes transactions in order: it starts from the user's opening balance, adds a top-up, then subtracts a purchase. The balance is updated in place using augmented assignment at each step.
+Write a program that reads the starting balance, the top-up amount, and the purchase amount, updates the balance with `balance += top_up` followed by `balance -= purchase`, and prints the final balance.
 ### Input Format
-- Line 1: Balance
-- Line 2: Deposit
-- Line 3: Expense
+- Line 1: Starting balance
+- Line 2: Top-up amount
+- Line 3: Purchase amount
 ### Output Format
 ```
 125.0
 ```
+### Example Walkthrough
+In the sample, the balance starts at 100. Adding a top-up of 50 makes it 150, then subtracting a purchase of 25 makes it 125.0, which the program prints.
 ### Constraints
-- Inputs follow the described format.
-- Print exactly the requested output with no extra text.</t>
+- All numeric inputs are valid numbers in the ranges implied by the examples.
+- Every value must be printed exactly as shown in the output format, with no extra text added or removed.</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -7830,17 +7854,21 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>A supplemental Python practice task for Gate Pass Boolean. Read the input values and print the required result exactly.
+          <t>A hostel's visitor gate pass system only issues a pass automatically when a visitor is an adult (18 years or older) AND has already paid the entry fee at the counter. The security guard's tablet reads both pieces of information and shows whether the pass should be granted.
+Write a program that reads the visitor's age and whether they have paid (`True` or `False`), then prints `True` if the visitor is 18 or older AND has paid, and `False` otherwise.
 ### Input Format
 - Line 1: Age
-- Line 2: True/False paid
+- Line 2: `True` or `False` indicating whether the visitor has paid
 ### Output Format
 ```
 True
 ```
+### Example Walkthrough
+In the sample, the age is 18 and paid is `True`. Since 18 is greater than or equal to 18 and the visitor has paid, both conditions are true, so the program prints `True`.
 ### Constraints
-- Inputs follow the described format.
-- Print exactly the requested output with no extra text.</t>
+- Age is a valid whole number in the ranges implied by the examples.
+- The paid input is always exactly `True` or `False`.
+- Every value must be printed exactly as shown in the output format, with no extra text added or removed.</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -7993,18 +8021,21 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>A supplemental Python practice task for Cast Sum Product. Read the input values and print the required result exactly.
+          <t>A calculator widget lets a user type two numbers into text boxes, but every value read from a text box arrives as a string. Before the widget can do any arithmetic, it must convert each entry to an integer.
+Write a program that reads two whole numbers (converting each from text to an integer), then prints their sum and product on separate lines in the form `Sum: &lt;value&gt;` and `Product: &lt;value&gt;`.
 ### Input Format
-- Line 1: First
-- Line 2: Second
+- Line 1: First number
+- Line 2: Second number
 ### Output Format
 ```
 Sum: 5
 Product: 6
 ```
+### Example Walkthrough
+In the sample, the numbers are 2 and 3. Converting both to integers and computing gives a sum of 2 + 3 = 5 and a product of 2 x 3 = 6, so the program prints `Sum: 5` and `Product: 6`.
 ### Constraints
-- Inputs follow the described format.
-- Print exactly the requested output with no extra text.</t>
+- All numeric inputs are valid whole numbers in the ranges implied by the examples.
+- Every value must be printed exactly as shown in the output format, with no extra text added or removed.</t>
         </is>
       </c>
       <c r="D11" t="n">

</xml_diff>